<commit_message>
Fix subdiv-matched english leaking into Review/Unmatched
- An english name claimed by subdivision discovery (e.g. Kab Elias ->
  قب الياس التحتا/الفوقا) kept its review candidates and unmatched row
- Add decided_en = auto | suggested | subdiv; exclude from Review sheet,
  Unmatched sheet, and 'still unmatched' / review summary counts
- Regenerated workbook + docs/data.json: review 70->69, unmatched EN 398->397
</commit_message>
<xml_diff>
--- a/FuzzyMatch/Lebanese_Villages_Matched_v6.xlsx
+++ b/FuzzyMatch/Lebanese_Villages_Matched_v6.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="18">
@@ -80241,7 +80241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81209,29 +81209,29 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kab Elias</t>
+          <t>Kaoutarite El-Riz</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Zahleh</t>
+          <t>Saida</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Bekaa</t>
+          <t>South</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>كابوسية (زحلة) [75.0]</t>
+          <t>القنيطرة (قرى صيدا) [77.1]</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kaoutarite El-Riz</t>
+          <t>Kaoutarite El-Siyad</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -81246,63 +81246,68 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>القنيطرة (قرى صيدا) [77.1]</t>
+          <t>كوثرية السياد (قرى صيدا) [82.4]</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kaoutarite El-Siyad</t>
+          <t>Katté</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Saida</t>
+          <t>Akkar</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Akkar</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>كوثرية السياد (قرى صيدا) [82.4]</t>
+          <t>البقيعة (عكار) [75.0]</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Katté</t>
+          <t>Kfar-Mashoune et Dmalsa</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Akkar</t>
+          <t>Jubail</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Akkar</t>
+          <t>Mount Lebanon</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>البقيعة (عكار) [75.0]</t>
+          <t>كفر مسحون (جبيل) [80.0]</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>مزرعة السياد (جبيل) [72.0]</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kfar-Mashoune et Dmalsa</t>
+          <t>Kobbaï</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Jubail</t>
+          <t>Baabda</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -81312,46 +81317,41 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>كفر مسحون (جبيل) [80.0]</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>مزرعة السياد (جبيل) [72.0]</t>
+          <t>قبيع (بعبدا) [75.0]</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kobbaï</t>
+          <t>Lebaa</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Baabda</t>
+          <t>Jezzine</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mount Lebanon</t>
+          <t>South</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>قبيع (بعبدا) [75.0]</t>
+          <t>لبعه (جزين) [85.7]</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Lebaa</t>
+          <t>Mazraat Dhaira</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jezzine</t>
+          <t>Sour</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -81361,14 +81361,14 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>لبعه (جزين) [85.7]</t>
+          <t>الظهيرة (صور) [72.7]</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mazraat Dhaira</t>
+          <t>Mazraat Ez-Zalloutieh</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -81383,36 +81383,36 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>الظهيرة (صور) [72.7]</t>
+          <t>الزلوطية (صور) [77.1]</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Mazraat Ez-Zalloutieh</t>
+          <t>Mazraet-el-Siyad</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Sour</t>
+          <t>Jubail</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Mount Lebanon</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>الزلوطية (صور) [77.1]</t>
+          <t>مزرعة السياد (جبيل) [72.7]</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Mazraet-el-Siyad</t>
+          <t>Mechmech</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -81427,14 +81427,14 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>مزرعة السياد (جبيل) [72.7]</t>
+          <t>كفر مسحون (جبيل) [77.1]</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mechmech</t>
+          <t>Mehrine</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -81449,107 +81449,107 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>كفر مسحون (جبيل) [77.1]</t>
+          <t>كفر مسحون (جبيل) [75.0]</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mehrine</t>
+          <t>Merh Kfarsghabe</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jubail</t>
+          <t>Zgharta</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Mount Lebanon</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>كفر مسحون (جبيل) [75.0]</t>
+          <t>مزرعة حوقا (زغرتا) [72.0]</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Merh Kfarsghabe</t>
+          <t>Michaa Mrajhiné</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Zgharta</t>
+          <t>Hermel</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Baalbak - Hermel</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>مزرعة حوقا (زغرتا) [72.0]</t>
+          <t>مراح العين (قضاءي بعلبك والهرمل) [72.0]</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Michaa Mrajhiné</t>
+          <t>Miemié</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Hermel</t>
+          <t>Saida</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Baalbak - Hermel</t>
+          <t>South</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>مراح العين (قضاءي بعلبك والهرمل) [72.0]</t>
+          <t>المية ومية (قرى صيدا) [72.7]</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Miemié</t>
+          <t>Mrabine</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Saida</t>
+          <t>Minieh-Danieh</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>المية ومية (قرى صيدا) [72.7]</t>
+          <t>نمرين (الضنية) [75.0]</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Mrabine</t>
+          <t>Mugher-el-Ahwel</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Minieh-Danieh</t>
+          <t>Bcharre</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -81559,41 +81559,46 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>نمرين (الضنية) [75.0]</t>
+          <t>المغر وبلا (بشري) [85.7]</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Mugher-el-Ahwel</t>
+          <t>Naamat</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Bcharre</t>
+          <t>Chouf</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Mount Lebanon</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>المغر وبلا (بشري) [85.7]</t>
+          <t>الناعمه (الشوف) [80.0]</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>حارة الناعمه (الشوف) [72.0]</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Naamat</t>
+          <t>Nammoura et Kfar Jerif</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Chouf</t>
+          <t>Kasrouane</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -81603,41 +81608,46 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>الناعمه (الشوف) [80.0]</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>حارة الناعمه (الشوف) [72.0]</t>
+          <t>النموره وكفر جريف (كسروان) [80.0]</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Nammoura et Kfar Jerif</t>
+          <t>Ouadi El-Osse</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Kasrouane</t>
+          <t>Hermel</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Mount Lebanon</t>
+          <t>Baalbak - Hermel</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>النموره وكفر جريف (كسروان) [80.0]</t>
+          <t>وادي الصفا الشرقي (قضاءي بعلبك والهرمل) [85.5]</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>وادي المشمشه (قضاءي بعلبك والهرمل) [85.5]</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>وادي النيرة (قضاءي بعلبك والهرمل) [85.5]</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ouadi El-Osse</t>
+          <t>Ras Baalbek El-Gharbi</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -81652,24 +81662,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>وادي الصفا الشرقي (قضاءي بعلبك والهرمل) [85.5]</t>
+          <t>قلعة غربي (قضاءي بعلبك والهرمل) [81.8]</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>وادي المشمشه (قضاءي بعلبك والهرمل) [85.5]</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>وادي النيرة (قضاءي بعلبك والهرمل) [85.5]</t>
+          <t>الريش حي الغربي (قضاءي بعلبك والهرمل) [77.8]</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Ras Baalbek El-Gharbi</t>
+          <t>Ras-Baalbek - Wadi Faara</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -81684,56 +81689,51 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>قلعة غربي (قضاءي بعلبك والهرمل) [81.8]</t>
+          <t>وادي التركمان (قضاءي بعلبك والهرمل) [85.5]</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>الريش حي الغربي (قضاءي بعلبك والهرمل) [77.8]</t>
+          <t>وادي الرطل (قضاءي بعلبك والهرمل) [85.5]</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>وادي المشمشه (قضاءي بعلبك والهرمل) [85.5]</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Ras-Baalbek - Wadi Faara</t>
+          <t>Sarhita</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Hermel</t>
+          <t>Jubail</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Baalbak - Hermel</t>
+          <t>Mount Lebanon</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>وادي التركمان (قضاءي بعلبك والهرمل) [85.5]</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>وادي الرطل (قضاءي بعلبك والهرمل) [85.5]</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>وادي المشمشه (قضاءي بعلبك والهرمل) [85.5]</t>
+          <t>سرعيتا (جبيل) [76.9]</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Sarhita</t>
+          <t>Souhailet El-Faouka</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Jubail</t>
+          <t>Kasrouane</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -81743,107 +81743,107 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>سرعيتا (جبيل) [76.9]</t>
+          <t>السهيله (كسروان) [77.1]</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ساحل علما (كسروان) [77.1]</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Souhailet El-Faouka</t>
+          <t>Tal Sibhel</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Kasrouane</t>
+          <t>Akkar</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Mount Lebanon</t>
+          <t>Akkar</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>السهيله (كسروان) [77.1]</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>ساحل علما (كسروان) [77.1]</t>
+          <t>القبيات القطلبه (عكار) [72.0]</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Tal Sibhel</t>
+          <t>Tripoli Al-Mouhaitra</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Akkar</t>
+          <t>Tripoli</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Akkar</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>القبيات القطلبه (عكار) [72.0]</t>
+          <t>المهاترة (مدينة طرابلس) [80.0]</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Tripoli Al-Mouhaitra</t>
+          <t>Wadi Abou Youssef</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Tripoli</t>
+          <t>Chouf</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Mount Lebanon</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>المهاترة (مدينة طرابلس) [80.0]</t>
+          <t>وادي دير دوريت (الشوف) [85.5]</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Wadi Abou Youssef</t>
+          <t>Wadi-el-Arayeche</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Chouf</t>
+          <t>Zahleh</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Mount Lebanon</t>
+          <t>Bekaa</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>وادي دير دوريت (الشوف) [85.5]</t>
+          <t>زحلة وادي العرايش (زحلة) [85.5]</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Wadi-el-Arayeche</t>
+          <t>Zahlé (Terres)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -81858,14 +81858,14 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>زحلة وادي العرايش (زحلة) [85.5]</t>
+          <t>زحلة وادي العرايش (زحلة) [85.7]</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Zahlé (Terres)</t>
+          <t>Zahlé Maallaka Kerek</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -81880,37 +81880,15 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>زحلة وادي العرايش (زحلة) [85.7]</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Zahlé Maallaka Kerek</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Zahleh</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Bekaa</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
           <t>زحلة المعلقه (زحلة) [85.7]</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>زحلة كرك نوح (زحلة) [80.0]</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>زحلة المعلقه الشمالي (زحلة) [77.1]</t>
         </is>
@@ -81927,7 +81905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D696"/>
+  <dimension ref="A1:D695"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90034,7 +90012,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Kab Elias</t>
+          <t>Ksara</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -90056,7 +90034,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Ksara</t>
+          <t>Maallaka (Terres)</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -90078,7 +90056,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Maallaka (Terres)</t>
+          <t>Maazraat-el-Ramtanieh</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -90100,7 +90078,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Maazraat-el-Ramtanieh</t>
+          <t>Mandara</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -90122,7 +90100,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Mandara</t>
+          <t>Mejdel-Anjar</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -90144,7 +90122,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Mejdel-Anjar</t>
+          <t>Nasriyat Rizk</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -90166,7 +90144,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Nasriyat Rizk</t>
+          <t>Tal-al-Amara</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -90188,7 +90166,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Tal-al-Amara</t>
+          <t>Tchiflik Eddé</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -90210,7 +90188,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Tchiflik Eddé</t>
+          <t>Tchiflik Kikano</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -90232,7 +90210,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>Tchiflik Kikano</t>
+          <t>Wadi-el-Arayeche</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -90254,7 +90232,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>Wadi-el-Arayeche</t>
+          <t>Zahlé (Terres)</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -90276,7 +90254,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>Zahlé (Terres)</t>
+          <t>Zahlé Maallaka Kerek</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -90298,7 +90276,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>Zahlé Maallaka Kerek</t>
+          <t>Zahlé Mar Gérios</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -90320,7 +90298,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Zahlé Mar Gérios</t>
+          <t>Zebdol</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -90342,17 +90320,17 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Zebdol</t>
+          <t>Aadoua</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Zahleh</t>
+          <t>Zgharta</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>Bekaa</t>
+          <t>North</t>
         </is>
       </c>
     </row>
@@ -90364,7 +90342,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Aadoua</t>
+          <t>Al-Harik</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -90386,7 +90364,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Al-Harik</t>
+          <t>Al-Jdeidé</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -90408,7 +90386,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Al-Jdeidé</t>
+          <t>Al-Khaldyé</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -90430,7 +90408,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Al-Khaldyé</t>
+          <t>Arbet Koshaya</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -90452,7 +90430,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Arbet Koshaya</t>
+          <t>Ardate</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -90474,7 +90452,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Ardate</t>
+          <t>Bsebhil</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -90496,7 +90474,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Bsebhil</t>
+          <t>Danhi</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
@@ -90518,7 +90496,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Danhi</t>
+          <t>Ehden</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -90540,7 +90518,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Ehden</t>
+          <t>Ejbeh</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
@@ -90562,7 +90540,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Ejbeh</t>
+          <t>El-Tellé</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -90584,7 +90562,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>El-Tellé</t>
+          <t>Mazraat Ejbeh</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -90606,7 +90584,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Mazraat Ejbeh</t>
+          <t>Mazraat Jneide</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -90628,7 +90606,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Mazraat Jneide</t>
+          <t>Mejdlaya</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -90650,7 +90628,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Mejdlaya</t>
+          <t>Merh Kfarsghabe</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -90672,7 +90650,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Merh Kfarsghabe</t>
+          <t>Sakhra</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -90689,22 +90667,22 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Sakhra</t>
+          <t>راشكده</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Zgharta</t>
+          <t>البترون</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>الشمال</t>
         </is>
       </c>
     </row>
@@ -90716,7 +90694,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>راشكده</t>
+          <t>عورا</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -90738,7 +90716,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>عورا</t>
+          <t>غوما</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -90760,7 +90738,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>غوما</t>
+          <t>قندولا</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -90782,17 +90760,17 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>قندولا</t>
+          <t>الدبية</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>البترون</t>
+          <t>الشوف</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>الشمال</t>
+          <t>جبل لبنان</t>
         </is>
       </c>
     </row>
@@ -90804,7 +90782,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>الدبية</t>
+          <t>المحتقره دير المخلص</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -90826,7 +90804,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>المحتقره دير المخلص</t>
+          <t>الناعمه</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -90848,7 +90826,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>الناعمه</t>
+          <t>بقعاتا</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -90870,7 +90848,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>بقعاتا</t>
+          <t>جديدة الشوف</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -90892,7 +90870,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>جديدة الشوف</t>
+          <t>حارة الناعمه</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -90914,7 +90892,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>حارة الناعمه</t>
+          <t>حارة بعاصير</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -90936,7 +90914,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>حارة بعاصير</t>
+          <t>عين الاسد والشميس</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -90958,7 +90936,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>عين الاسد والشميس</t>
+          <t>عين الحور</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -90980,7 +90958,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>عين الحور</t>
+          <t>كليليه</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -91002,7 +90980,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>كليليه</t>
+          <t>مرج برجا</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -91024,7 +91002,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>مرج برجا</t>
+          <t>وادي دير دوريت</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -91046,17 +91024,17 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>وادي دير دوريت</t>
+          <t>الروضة</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>الشوف</t>
+          <t>الضنية</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>جبل لبنان</t>
+          <t>الشمال</t>
         </is>
       </c>
     </row>
@@ -91068,7 +91046,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>الروضة</t>
+          <t>المطل</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -91090,7 +91068,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>المطل</t>
+          <t>حرف السياد</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -91112,7 +91090,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>حرف السياد</t>
+          <t>عزقي</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -91134,7 +91112,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>عزقي</t>
+          <t>قزحيا</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -91156,7 +91134,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>قزحيا</t>
+          <t>كرم المهر</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -91178,7 +91156,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>كرم المهر</t>
+          <t>كفربنين</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -91200,7 +91178,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>كفربنين</t>
+          <t>نمرين</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -91222,12 +91200,12 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>نمرين</t>
+          <t>البحصاص</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>الضنية</t>
+          <t>الكورة</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
@@ -91244,7 +91222,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>البحصاص</t>
+          <t>حارة الخاصة</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -91266,7 +91244,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>حارة الخاصة</t>
+          <t>ضهر العين</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -91288,7 +91266,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>ضهر العين</t>
+          <t>ضهور الهوا</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -91310,17 +91288,17 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>ضهور الهوا</t>
+          <t>الرابية</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>الكورة</t>
+          <t>المتن</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>الشمال</t>
+          <t>جبل لبنان</t>
         </is>
       </c>
     </row>
@@ -91332,7 +91310,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>الرابية</t>
+          <t>سد البوشريه</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -91354,7 +91332,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>سد البوشريه</t>
+          <t>مزرعة بنابيل</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -91376,17 +91354,17 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>مزرعة بنابيل</t>
+          <t>المنية</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>المتن</t>
+          <t>المنية</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>جبل لبنان</t>
+          <t>الشمال</t>
         </is>
       </c>
     </row>
@@ -91398,17 +91376,17 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>المنية</t>
+          <t>كفروة</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>المنية</t>
+          <t>النبطية</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>الشمال</t>
+          <t>النبطية</t>
         </is>
       </c>
     </row>
@@ -91420,17 +91398,17 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>كفروة</t>
+          <t>المغر وبلا</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>النبطية</t>
+          <t>بشري</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>النبطية</t>
+          <t>الشمال</t>
         </is>
       </c>
     </row>
@@ -91442,17 +91420,17 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>المغر وبلا</t>
+          <t>الحدث شمالي</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>بشري</t>
+          <t>بعبدا</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>الشمال</t>
+          <t>جبل لبنان</t>
         </is>
       </c>
     </row>
@@ -91464,7 +91442,7 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>الحدث شمالي</t>
+          <t>الحدث قبلي</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -91486,7 +91464,7 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>الحدث قبلي</t>
+          <t>الشياح حي الكنيسة</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
@@ -91508,7 +91486,7 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>الشياح حي الكنيسة</t>
+          <t>الشياح حي كرم الزيتون</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
@@ -91530,7 +91508,7 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>الشياح حي كرم الزيتون</t>
+          <t>الغبيري بئر حسن</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
@@ -91552,7 +91530,7 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>الغبيري بئر حسن</t>
+          <t>الغبيري حي الجامع</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
@@ -91574,7 +91552,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>الغبيري حي الجامع</t>
+          <t>الفياضية</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
@@ -91596,7 +91574,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>الفياضية</t>
+          <t>القلعه</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -91618,7 +91596,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>القلعه</t>
+          <t>المريجه</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -91640,7 +91618,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>المريجه</t>
+          <t>تحويطة النهر</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -91662,7 +91640,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>تحويطة النهر</t>
+          <t>حارة البطم</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -91684,7 +91662,7 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>حارة البطم</t>
+          <t>حارة حريك قرانوح</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
@@ -91706,7 +91684,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>حارة حريك قرانوح</t>
+          <t>دير مار الياس الكحلونية</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -91728,7 +91706,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>دير مار الياس الكحلونية</t>
+          <t>سبنيه</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -91750,7 +91728,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>سبنيه</t>
+          <t>قبيع</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -91772,17 +91750,17 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>قبيع</t>
+          <t>حداثا</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>بعبدا</t>
+          <t>بنت جبيل</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>جبل لبنان</t>
+          <t>النبطية</t>
         </is>
       </c>
     </row>
@@ -91794,7 +91772,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>حداثا</t>
+          <t>عيتا الجبل</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -91816,17 +91794,17 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>عيتا الجبل</t>
+          <t>الجليسه</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>بنت جبيل</t>
+          <t>جبيل</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>النبطية</t>
+          <t>جبل لبنان</t>
         </is>
       </c>
     </row>
@@ -91838,7 +91816,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>الجليسه</t>
+          <t>العاقورة - م</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -91860,7 +91838,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>العاقورة - م</t>
+          <t>الفيدار</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
@@ -91882,7 +91860,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>الفيدار</t>
+          <t>المزاريب</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
@@ -91904,7 +91882,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>المزاريب</t>
+          <t>المنصف</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
@@ -91926,7 +91904,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>المنصف</t>
+          <t>بنتاعل</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
@@ -91948,7 +91926,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>بنتاعل</t>
+          <t>دملصا</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
@@ -91970,7 +91948,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>دملصا</t>
+          <t>دير القطاره</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
@@ -91992,7 +91970,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>دير القطاره</t>
+          <t>سرعيتا</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -92014,7 +91992,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>سرعيتا</t>
+          <t>عين الدلبة</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -92036,7 +92014,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>عين الدلبة</t>
+          <t>عين الشلال</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
@@ -92058,7 +92036,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>عين الشلال</t>
+          <t>عين الغويبة</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -92080,7 +92058,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>عين الغويبة</t>
+          <t>قرطبا الشمالية</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
@@ -92102,7 +92080,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>قرطبا الشمالية</t>
+          <t>كفر مسحون</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
@@ -92124,7 +92102,7 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>كفر مسحون</t>
+          <t>مزرعة السياد</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
@@ -92146,17 +92124,17 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>مزرعة السياد</t>
+          <t>بحنين - كفرتعلا</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>جبيل</t>
+          <t>جزين</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>جبل لبنان</t>
+          <t>الجنوب</t>
         </is>
       </c>
     </row>
@@ -92168,7 +92146,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>بحنين - كفرتعلا</t>
+          <t>عين مجدلين</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
@@ -92190,7 +92168,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>عين مجدلين</t>
+          <t>قتالة</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
@@ -92212,7 +92190,7 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>قتالة</t>
+          <t>لبعه</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
@@ -92234,17 +92212,17 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>لبعه</t>
+          <t>الكرمة</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>جزين</t>
+          <t>زحلة</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>الجنوب</t>
+          <t>البقاع</t>
         </is>
       </c>
     </row>
@@ -92256,7 +92234,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>الكرمة</t>
+          <t>بتياس</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
@@ -92278,7 +92256,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>بتياس</t>
+          <t>جلالا</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
@@ -92300,7 +92278,7 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>جلالا</t>
+          <t>حاجي حببلي</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
@@ -92322,7 +92300,7 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>حاجي حببلي</t>
+          <t>حي السلم</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
@@ -92344,7 +92322,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>حي السلم</t>
+          <t>حي الفيكاني</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
@@ -92366,7 +92344,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>حي الفيكاني</t>
+          <t>خضر بك</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
@@ -92388,7 +92366,7 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>خضر بك</t>
+          <t>زحلة المعلقه</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
@@ -92410,7 +92388,7 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>زحلة المعلقه</t>
+          <t>زحلة المعلقه الشمالي</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
@@ -92432,7 +92410,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>زحلة المعلقه الشمالي</t>
+          <t>زحلة حي السيدة</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
@@ -92454,7 +92432,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>زحلة حي السيدة</t>
+          <t>زحلة كرك نوح</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
@@ -92476,7 +92454,7 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>زحلة كرك نوح</t>
+          <t>زحلة مار مخايل</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
@@ -92498,7 +92476,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>زحلة مار مخايل</t>
+          <t>زحلة وادي العرايش</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
@@ -92520,7 +92498,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>زحلة وادي العرايش</t>
+          <t>شهابية الفاعور</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
@@ -92542,7 +92520,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>شهابية الفاعور</t>
+          <t>كابوسية</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
@@ -92564,7 +92542,7 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>كابوسية</t>
+          <t>يوغون اولوك</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
@@ -92586,17 +92564,17 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>يوغون اولوك</t>
+          <t>اجبع</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>زحلة</t>
+          <t>زغرتا</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>البقاع</t>
+          <t>الشمال</t>
         </is>
       </c>
     </row>
@@ -92608,7 +92586,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>اجبع</t>
+          <t>اسلوت</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
@@ -92630,7 +92608,7 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>اسلوت</t>
+          <t>القادريه</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
@@ -92652,7 +92630,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>القادريه</t>
+          <t>بيت عبيد</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -92674,7 +92652,7 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>بيت عبيد</t>
+          <t>بيت عوكر</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
@@ -92696,7 +92674,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>بيت عوكر</t>
+          <t>حارة الفوار</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
@@ -92718,7 +92696,7 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>حارة الفوار</t>
+          <t>حرف ارده</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
@@ -92740,7 +92718,7 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>حرف ارده</t>
+          <t>حرف مزيارة</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
@@ -92762,7 +92740,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>حرف مزيارة</t>
+          <t>عربة قزحيا</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
@@ -92784,7 +92762,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>عربة قزحيا</t>
+          <t>مزرعة الفريديس</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
@@ -92806,7 +92784,7 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>مزرعة الفريديس</t>
+          <t>مزرعة حوقا</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
@@ -92828,17 +92806,17 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>مزرعة حوقا</t>
+          <t>البازوريه</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>زغرتا</t>
+          <t>صور</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>الشمال</t>
+          <t>الجنوب</t>
         </is>
       </c>
     </row>
@@ -92850,7 +92828,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>البازوريه</t>
+          <t>البرغليه</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
@@ -92872,7 +92850,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>البرغليه</t>
+          <t>البساتين</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
@@ -92894,7 +92872,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>البساتين</t>
+          <t>البص  قسم 1</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
@@ -92916,7 +92894,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>البص  قسم 1</t>
+          <t>البص  قسم 3</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
@@ -92938,7 +92916,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>البص  قسم 3</t>
+          <t>البص قسم 5</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
@@ -92960,7 +92938,7 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>البص قسم 5</t>
+          <t>الحميري</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
@@ -92982,7 +92960,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>الحميري</t>
+          <t>الرشيديه</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
@@ -93004,7 +92982,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>الرشيديه</t>
+          <t>الزلوطية</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
@@ -93026,7 +93004,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>الزلوطية</t>
+          <t>السماعية</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
@@ -93048,7 +93026,7 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>السماعية</t>
+          <t>الشهابية</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
@@ -93070,7 +93048,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>الشهابية</t>
+          <t>الظهيرة</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
@@ -93092,7 +93070,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>الظهيرة</t>
+          <t>المالكية</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
@@ -93114,7 +93092,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>المالكية</t>
+          <t>بثتيات</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
@@ -93136,7 +93114,7 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>بثتيات</t>
+          <t>شبريحا</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
@@ -93158,7 +93136,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>شبريحا</t>
+          <t>شمع</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
@@ -93180,7 +93158,7 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>شمع</t>
+          <t>صور حي الارثوذكس</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
@@ -93202,7 +93180,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>صور حي الارثوذكس</t>
+          <t>صور حي الجامع</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
@@ -93224,7 +93202,7 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>صور حي الجامع</t>
+          <t>صور حي الجورة</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
@@ -93246,7 +93224,7 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>صور حي الجورة</t>
+          <t>صور حي الحسينية</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
@@ -93268,7 +93246,7 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>صور حي الحسينية</t>
+          <t>صور حي الكاثوليك</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
@@ -93290,7 +93268,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>صور حي الكاثوليك</t>
+          <t>صور حي المصاروي</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
@@ -93312,7 +93290,7 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>صور حي المصاروي</t>
+          <t>صور حي المنارة</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
@@ -93334,7 +93312,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>صور حي المنارة</t>
+          <t>صور حي الموارنة</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -93356,7 +93334,7 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>صور حي الموارنة</t>
+          <t>عين الزرقا</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
@@ -93378,7 +93356,7 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>عين الزرقا</t>
+          <t>محرونه</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
@@ -93400,17 +93378,17 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>محرونه</t>
+          <t>البساتين</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>صور</t>
+          <t>عاليه</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>الجنوب</t>
+          <t>جبل لبنان</t>
         </is>
       </c>
     </row>
@@ -93422,7 +93400,7 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>البساتين</t>
+          <t>التعزانية</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
@@ -93444,7 +93422,7 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>التعزانية</t>
+          <t>جسر القاضي</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
@@ -93466,7 +93444,7 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>جسر القاضي</t>
+          <t>عاليه قبلي</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
@@ -93488,7 +93466,7 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>عاليه قبلي</t>
+          <t>عاليه وسطاني</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
@@ -93510,7 +93488,7 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>عاليه وسطاني</t>
+          <t>عين الفريديس</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
@@ -93532,7 +93510,7 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>عين الفريديس</t>
+          <t>محطة بحمدون</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
@@ -93554,17 +93532,17 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>محطة بحمدون</t>
+          <t>البساتين</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>عاليه</t>
+          <t>عكار</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>جبل لبنان</t>
+          <t>عكار</t>
         </is>
       </c>
     </row>
@@ -93576,7 +93554,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>البساتين</t>
+          <t>البقيعة</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
@@ -93598,7 +93576,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>البقيعة</t>
+          <t>الحويش</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
@@ -93620,7 +93598,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>الحويش</t>
+          <t>الدوسه</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
@@ -93642,7 +93620,7 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>الدوسه</t>
+          <t>السهلة</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
@@ -93664,7 +93642,7 @@
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>السهلة</t>
+          <t>الشيخ عياش</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
@@ -93686,7 +93664,7 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>الشيخ عياش</t>
+          <t>العماير</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
@@ -93708,7 +93686,7 @@
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>العماير</t>
+          <t>العوادة</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
@@ -93730,7 +93708,7 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>العوادة</t>
+          <t>الفرض</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
@@ -93752,7 +93730,7 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>الفرض</t>
+          <t>القبيات الذوق</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
@@ -93774,7 +93752,7 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>القبيات الذوق</t>
+          <t>القبيات الضهر</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
@@ -93796,7 +93774,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>القبيات الضهر</t>
+          <t>القبيات الغربية</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
@@ -93818,7 +93796,7 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>القبيات الغربية</t>
+          <t>القبيات القطلبه</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
@@ -93840,7 +93818,7 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>القبيات القطلبه</t>
+          <t>القبيات غوايا</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
@@ -93862,7 +93840,7 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>القبيات غوايا</t>
+          <t>القبيات مرتموره</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
@@ -93884,7 +93862,7 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>القبيات مرتموره</t>
+          <t>المونسة</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
@@ -93906,7 +93884,7 @@
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>المونسة</t>
+          <t>الهيشة</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
@@ -93928,7 +93906,7 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>الهيشة</t>
+          <t>برج العرب</t>
         </is>
       </c>
       <c r="C546" t="inlineStr">
@@ -93950,7 +93928,7 @@
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>برج العرب</t>
+          <t>بني صخر</t>
         </is>
       </c>
       <c r="C547" t="inlineStr">
@@ -93972,7 +93950,7 @@
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>بني صخر</t>
+          <t>بيت الحاج</t>
         </is>
       </c>
       <c r="C548" t="inlineStr">
@@ -93994,7 +93972,7 @@
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>بيت الحاج</t>
+          <t>تل معيان</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
@@ -94016,7 +93994,7 @@
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>تل معيان</t>
+          <t>تلبيبة</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
@@ -94038,7 +94016,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>تلبيبة</t>
+          <t>جبل المنصورة</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
@@ -94060,7 +94038,7 @@
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>جبل المنصورة</t>
+          <t>جرمنايا</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
@@ -94082,7 +94060,7 @@
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>جرمنايا</t>
+          <t>خربة الجرد</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
@@ -94104,7 +94082,7 @@
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>خربة الجرد</t>
+          <t>خريبة الجندي</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
@@ -94126,7 +94104,7 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>خريبة الجندي</t>
+          <t>خط البترول</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
@@ -94148,7 +94126,7 @@
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>خط البترول</t>
+          <t>رجم عيسى</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
@@ -94170,7 +94148,7 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>رجم عيسى</t>
+          <t>ضهر القنبر</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
@@ -94192,7 +94170,7 @@
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>ضهر القنبر</t>
+          <t>عبودية</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
@@ -94214,7 +94192,7 @@
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>عبودية</t>
+          <t>عين الذهب</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
@@ -94236,7 +94214,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>عين الذهب</t>
+          <t>قنية</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
@@ -94258,7 +94236,7 @@
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>قنية</t>
+          <t>كرم زبدين</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
@@ -94280,7 +94258,7 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>كرم زبدين</t>
+          <t>مراح الخوخ</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
@@ -94302,17 +94280,17 @@
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>مراح الخوخ</t>
+          <t>الحجة</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>عكار</t>
+          <t>قرى صيدا</t>
         </is>
       </c>
       <c r="D563" t="inlineStr">
         <is>
-          <t>عكار</t>
+          <t>الجنوب</t>
         </is>
       </c>
     </row>
@@ -94324,7 +94302,7 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>الحجة</t>
+          <t>القنيطرة</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
@@ -94346,7 +94324,7 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>القنيطرة</t>
+          <t>المعمرية</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
@@ -94368,7 +94346,7 @@
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>المعمرية</t>
+          <t>المية ومية</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
@@ -94390,7 +94368,7 @@
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>المية ومية</t>
+          <t>كوثرية السياد</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
@@ -94412,17 +94390,17 @@
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>كوثرية السياد</t>
+          <t>الروضة</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>قرى صيدا</t>
+          <t>قضاءي البقاع الغربي وراشيا</t>
         </is>
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>الجنوب</t>
+          <t>البقاع</t>
         </is>
       </c>
     </row>
@@ -94434,7 +94412,7 @@
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>الروضة</t>
+          <t>الشبرقية</t>
         </is>
       </c>
       <c r="C569" t="inlineStr">
@@ -94456,7 +94434,7 @@
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>الشبرقية</t>
+          <t>دير العشائر</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
@@ -94478,7 +94456,7 @@
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>دير العشائر</t>
+          <t>راشيا حي الفوقا</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
@@ -94500,7 +94478,7 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>راشيا حي الفوقا</t>
+          <t>راشيا حي الكواسبه</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
@@ -94522,7 +94500,7 @@
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>راشيا حي الكواسبه</t>
+          <t>راشيا حي الميدان</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
@@ -94544,7 +94522,7 @@
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>راشيا حي الميدان</t>
+          <t>عيحا</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
@@ -94566,7 +94544,7 @@
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>عيحا</t>
+          <t>عين التينه</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
@@ -94588,7 +94566,7 @@
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>عين التينه</t>
+          <t>كفردنيس</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
@@ -94610,7 +94588,7 @@
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>كفردنيس</t>
+          <t>كفرقوق</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
@@ -94632,7 +94610,7 @@
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>كفرقوق</t>
+          <t>محيدثه</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
@@ -94654,17 +94632,17 @@
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>محيدثه</t>
+          <t>الانصار</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>قضاءي البقاع الغربي وراشيا</t>
+          <t>قضاءي بعلبك والهرمل</t>
         </is>
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>البقاع</t>
+          <t>بعلبك والهرمل</t>
         </is>
       </c>
     </row>
@@ -94676,7 +94654,7 @@
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>الانصار</t>
+          <t>البرانيه حي المسيحيين</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
@@ -94698,7 +94676,7 @@
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>البرانيه حي المسيحيين</t>
+          <t>البرباره محلة المسيحيين</t>
         </is>
       </c>
       <c r="C581" t="inlineStr">
@@ -94720,7 +94698,7 @@
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>البرباره محلة المسيحيين</t>
+          <t>البويضة</t>
         </is>
       </c>
       <c r="C582" t="inlineStr">
@@ -94742,7 +94720,7 @@
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>البويضة</t>
+          <t>البويضة الحي الغربي</t>
         </is>
       </c>
       <c r="C583" t="inlineStr">
@@ -94764,7 +94742,7 @@
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>البويضة الحي الغربي</t>
+          <t>البويضة الشمالية</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
@@ -94786,7 +94764,7 @@
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>البويضة الشمالية</t>
+          <t>التوفيقيه</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
@@ -94808,7 +94786,7 @@
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>التوفيقيه</t>
+          <t>الجوبانية</t>
         </is>
       </c>
       <c r="C586" t="inlineStr">
@@ -94830,7 +94808,7 @@
       </c>
       <c r="B587" t="inlineStr">
         <is>
-          <t>الجوبانية</t>
+          <t>الحدث الشمالي</t>
         </is>
       </c>
       <c r="C587" t="inlineStr">
@@ -94852,7 +94830,7 @@
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>الحدث الشمالي</t>
+          <t>الحدث الغربي</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
@@ -94874,7 +94852,7 @@
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>الحدث الغربي</t>
+          <t>الحريقه</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
@@ -94896,7 +94874,7 @@
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>الحريقه</t>
+          <t>الحلانيه</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
@@ -94918,7 +94896,7 @@
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>الحلانيه</t>
+          <t>الخضر الشرقي</t>
         </is>
       </c>
       <c r="C591" t="inlineStr">
@@ -94940,7 +94918,7 @@
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>الخضر الشرقي</t>
+          <t>الخضر الغربي</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
@@ -94962,7 +94940,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>الخضر الغربي</t>
+          <t>الخضر حي الاشعل</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -94984,7 +94962,7 @@
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>الخضر حي الاشعل</t>
+          <t>الخضر حي الجنوبي</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
@@ -95006,7 +94984,7 @@
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>الخضر حي الجنوبي</t>
+          <t>الخضر حي الشعب</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -95028,7 +95006,7 @@
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>الخضر حي الشعب</t>
+          <t>الريش حي الشرقي</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
@@ -95050,7 +95028,7 @@
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>الريش حي الشرقي</t>
+          <t>الريش حي الشميس</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
@@ -95072,7 +95050,7 @@
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>الريش حي الشميس</t>
+          <t>الريش حي الغربي</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
@@ -95094,7 +95072,7 @@
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>الريش حي الغربي</t>
+          <t>الزرازير</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
@@ -95116,7 +95094,7 @@
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>الزرازير</t>
+          <t>الزويتيني</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
@@ -95138,7 +95116,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>الزويتيني</t>
+          <t>السعيده</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -95160,7 +95138,7 @@
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>السعيده</t>
+          <t>السويسة</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
@@ -95182,7 +95160,7 @@
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>السويسة</t>
+          <t>الشواغير التحتا</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
@@ -95204,7 +95182,7 @@
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>الشواغير التحتا</t>
+          <t>الشواغير الفوقا</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
@@ -95226,7 +95204,7 @@
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>الشواغير الفوقا</t>
+          <t>الصوانية</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
@@ -95248,7 +95226,7 @@
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>الصوانية</t>
+          <t>العقيدية</t>
         </is>
       </c>
       <c r="C606" t="inlineStr">
@@ -95270,7 +95248,7 @@
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>العقيدية</t>
+          <t>العلاق</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
@@ -95292,7 +95270,7 @@
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>العلاق</t>
+          <t>الفاكهة حي الجامع</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
@@ -95314,7 +95292,7 @@
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>الفاكهة حي الجامع</t>
+          <t>الفاكهة حي مار جرجس</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
@@ -95336,7 +95314,7 @@
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>الفاكهة حي مار جرجس</t>
+          <t>القاع</t>
         </is>
       </c>
       <c r="C610" t="inlineStr">
@@ -95358,7 +95336,7 @@
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>القاع</t>
+          <t>القدام</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
@@ -95380,7 +95358,7 @@
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>القدام</t>
+          <t>القرينة</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
@@ -95402,7 +95380,7 @@
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>القرينة</t>
+          <t>القصر</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
@@ -95424,7 +95402,7 @@
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>القصر</t>
+          <t>الكواخ</t>
         </is>
       </c>
       <c r="C614" t="inlineStr">
@@ -95446,7 +95424,7 @@
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>الكواخ</t>
+          <t>المعاصر</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
@@ -95468,7 +95446,7 @@
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>المعاصر</t>
+          <t>النبي رشاده</t>
         </is>
       </c>
       <c r="C616" t="inlineStr">
@@ -95490,7 +95468,7 @@
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>النبي رشاده</t>
+          <t>النبي شيت حي الجنوبي</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
@@ -95512,7 +95490,7 @@
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>النبي شيت حي الجنوبي</t>
+          <t>النبي شيت حي الشرقي</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
@@ -95534,7 +95512,7 @@
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>النبي شيت حي الشرقي</t>
+          <t>النبي شيت حي الشمالي</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
@@ -95556,7 +95534,7 @@
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>النبي شيت حي الشمالي</t>
+          <t>النبي شيت حي العريض</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
@@ -95578,7 +95556,7 @@
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>النبي شيت حي العريض</t>
+          <t>النبي شيت حي العقبة</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
@@ -95600,7 +95578,7 @@
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>النبي شيت حي العقبة</t>
+          <t>النبي شيت حي الغربي</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
@@ -95622,7 +95600,7 @@
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>النبي شيت حي الغربي</t>
+          <t>النبي شيت حي طبشار</t>
         </is>
       </c>
       <c r="C623" t="inlineStr">
@@ -95644,7 +95622,7 @@
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>النبي شيت حي طبشار</t>
+          <t>النبي نعام</t>
         </is>
       </c>
       <c r="C624" t="inlineStr">
@@ -95666,7 +95644,7 @@
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>النبي نعام</t>
+          <t>النقرة</t>
         </is>
       </c>
       <c r="C625" t="inlineStr">
@@ -95688,7 +95666,7 @@
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>النقرة</t>
+          <t>بريصا</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
@@ -95710,7 +95688,7 @@
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>بريصا</t>
+          <t>بيت ابو صليبي</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
@@ -95732,7 +95710,7 @@
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>بيت ابو صليبي</t>
+          <t>جوار الحشيش</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
@@ -95754,7 +95732,7 @@
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>جوار الحشيش</t>
+          <t>حوش السيد علي</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
@@ -95776,7 +95754,7 @@
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>حوش السيد علي</t>
+          <t>حي الزهراء</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
@@ -95798,7 +95776,7 @@
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>حي الزهراء</t>
+          <t>حي الصلح</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
@@ -95820,7 +95798,7 @@
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>حي الصلح</t>
+          <t>حي العباسية</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
@@ -95842,7 +95820,7 @@
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>حي العباسية</t>
+          <t>حي عز الدين</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
@@ -95864,7 +95842,7 @@
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>حي عز الدين</t>
+          <t>دار الواسعة</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
@@ -95886,7 +95864,7 @@
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>دار الواسعة</t>
+          <t>رماسا</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
@@ -95908,7 +95886,7 @@
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>رماسا</t>
+          <t>سهلات الماء</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
@@ -95930,7 +95908,7 @@
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>سهلات الماء</t>
+          <t>شعت حي الضهر</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
@@ -95952,7 +95930,7 @@
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>شعت حي الضهر</t>
+          <t>صفرا</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -95974,7 +95952,7 @@
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>صفرا</t>
+          <t>غفره</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
@@ -95996,7 +95974,7 @@
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>غفره</t>
+          <t>فلاوي</t>
         </is>
       </c>
       <c r="C640" t="inlineStr">
@@ -96018,7 +95996,7 @@
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>فلاوي</t>
+          <t>فيسان</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
@@ -96040,7 +96018,7 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>فيسان</t>
+          <t>قبة دورس</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -96062,7 +96040,7 @@
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>قبة دورس</t>
+          <t>قلد السبع</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -96084,7 +96062,7 @@
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>قلد السبع</t>
+          <t>قلعة</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
@@ -96106,7 +96084,7 @@
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>قلعة</t>
+          <t>قلعة غربي</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
@@ -96128,7 +96106,7 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>قلعة غربي</t>
+          <t>قنافذ</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
@@ -96150,7 +96128,7 @@
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>قنافذ</t>
+          <t>كفردبش</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
@@ -96172,7 +96150,7 @@
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>كفردبش</t>
+          <t>مراح العين</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
@@ -96194,7 +96172,7 @@
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>مراح العين</t>
+          <t>مزرعة آل سويدان</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
@@ -96216,7 +96194,7 @@
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>مزرعة آل سويدان</t>
+          <t>مزرعة ابو صليبي</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
@@ -96238,7 +96216,7 @@
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>مزرعة ابو صليبي</t>
+          <t>مزرعة التوت</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
@@ -96260,7 +96238,7 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>مزرعة التوت</t>
+          <t>مزرعة الضليل</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
@@ -96282,7 +96260,7 @@
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>مزرعة الضليل</t>
+          <t>مزرعة الفقيه</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
@@ -96304,7 +96282,7 @@
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>مزرعة الفقيه</t>
+          <t>مزرعة بيت الطشم</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
@@ -96326,7 +96304,7 @@
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>مزرعة بيت الطشم</t>
+          <t>مزرعة بيت مطر</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
@@ -96348,7 +96326,7 @@
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>مزرعة بيت مطر</t>
+          <t>مزرعة سجد</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
@@ -96370,7 +96348,7 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>مزرعة سجد</t>
+          <t>مصنع الزهرة</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
@@ -96392,7 +96370,7 @@
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>مصنع الزهرة</t>
+          <t>وادي التركمان</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
@@ -96414,7 +96392,7 @@
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>وادي التركمان</t>
+          <t>وادي الرطل</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
@@ -96436,7 +96414,7 @@
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>وادي الرطل</t>
+          <t>وادي الزين</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
@@ -96458,7 +96436,7 @@
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>وادي الزين</t>
+          <t>وادي الصفا الشرقي</t>
         </is>
       </c>
       <c r="C661" t="inlineStr">
@@ -96480,7 +96458,7 @@
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>وادي الصفا الشرقي</t>
+          <t>وادي المشمشه</t>
         </is>
       </c>
       <c r="C662" t="inlineStr">
@@ -96502,7 +96480,7 @@
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>وادي المشمشه</t>
+          <t>وادي النيرة</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
@@ -96524,7 +96502,7 @@
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>وادي النيرة</t>
+          <t>وادي بنيت</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
@@ -96546,17 +96524,17 @@
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>وادي بنيت</t>
+          <t>الجديدة حي السراي</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>قضاءي بعلبك والهرمل</t>
+          <t>قضاءي مرجعيون وحاصبيا</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>بعلبك والهرمل</t>
+          <t>النبطية</t>
         </is>
       </c>
     </row>
@@ -96568,7 +96546,7 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>الجديدة حي السراي</t>
+          <t>الجديدة حي العيون</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
@@ -96590,7 +96568,7 @@
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>الجديدة حي العيون</t>
+          <t>الجديدة حي القلعة</t>
         </is>
       </c>
       <c r="C667" t="inlineStr">
@@ -96612,7 +96590,7 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>الجديدة حي القلعة</t>
+          <t>الجديدة حي المدارس</t>
         </is>
       </c>
       <c r="C668" t="inlineStr">
@@ -96634,7 +96612,7 @@
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>الجديدة حي المدارس</t>
+          <t>الدلافة</t>
         </is>
       </c>
       <c r="C669" t="inlineStr">
@@ -96656,7 +96634,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>الدلافة</t>
+          <t>الفرديس</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
@@ -96678,7 +96656,7 @@
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>الفرديس</t>
+          <t>الهبارية</t>
         </is>
       </c>
       <c r="C671" t="inlineStr">
@@ -96700,7 +96678,7 @@
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>الهبارية</t>
+          <t>الوزاني</t>
         </is>
       </c>
       <c r="C672" t="inlineStr">
@@ -96722,7 +96700,7 @@
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>الوزاني</t>
+          <t>برج الملوك</t>
         </is>
       </c>
       <c r="C673" t="inlineStr">
@@ -96744,7 +96722,7 @@
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>برج الملوك</t>
+          <t>بويضة</t>
         </is>
       </c>
       <c r="C674" t="inlineStr">
@@ -96766,7 +96744,7 @@
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>بويضة</t>
+          <t>حاصبيا حي السراي</t>
         </is>
       </c>
       <c r="C675" t="inlineStr">
@@ -96788,7 +96766,7 @@
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>حاصبيا حي السراي</t>
+          <t>حاصبيا حي العين</t>
         </is>
       </c>
       <c r="C676" t="inlineStr">
@@ -96810,7 +96788,7 @@
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>حاصبيا حي العين</t>
+          <t>حاصبيا حي الفوقاني</t>
         </is>
       </c>
       <c r="C677" t="inlineStr">
@@ -96832,7 +96810,7 @@
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>حاصبيا حي الفوقاني</t>
+          <t>حاصبيا حي صفيفة</t>
         </is>
       </c>
       <c r="C678" t="inlineStr">
@@ -96854,7 +96832,7 @@
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>حاصبيا حي صفيفة</t>
+          <t>رب ثلاثين</t>
         </is>
       </c>
       <c r="C679" t="inlineStr">
@@ -96876,7 +96854,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>رب ثلاثين</t>
+          <t>سرده والعمره</t>
         </is>
       </c>
       <c r="C680" t="inlineStr">
@@ -96898,7 +96876,7 @@
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>سرده والعمره</t>
+          <t>عديسه</t>
         </is>
       </c>
       <c r="C681" t="inlineStr">
@@ -96920,7 +96898,7 @@
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>عديسه</t>
+          <t>كفرشوبا</t>
         </is>
       </c>
       <c r="C682" t="inlineStr">
@@ -96942,17 +96920,17 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>كفرشوبا</t>
+          <t>السهيله</t>
         </is>
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>قضاءي مرجعيون وحاصبيا</t>
+          <t>كسروان</t>
         </is>
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>النبطية</t>
+          <t>جبل لبنان</t>
         </is>
       </c>
     </row>
@@ -96964,7 +96942,7 @@
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>السهيله</t>
+          <t>النموره وكفر جريف</t>
         </is>
       </c>
       <c r="C684" t="inlineStr">
@@ -96986,7 +96964,7 @@
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>النموره وكفر جريف</t>
+          <t>ساحل علما</t>
         </is>
       </c>
       <c r="C685" t="inlineStr">
@@ -97008,7 +96986,7 @@
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>ساحل علما</t>
+          <t>شوان والعبره</t>
         </is>
       </c>
       <c r="C686" t="inlineStr">
@@ -97030,7 +97008,7 @@
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>شوان والعبره</t>
+          <t>غزير القناة</t>
         </is>
       </c>
       <c r="C687" t="inlineStr">
@@ -97052,7 +97030,7 @@
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>غزير القناة</t>
+          <t>غزير المعاملتين</t>
         </is>
       </c>
       <c r="C688" t="inlineStr">
@@ -97074,17 +97052,17 @@
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>غزير المعاملتين</t>
+          <t>التبانة</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>كسروان</t>
+          <t>مدينة طرابلس</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
         <is>
-          <t>جبل لبنان</t>
+          <t>الشمال</t>
         </is>
       </c>
     </row>
@@ -97096,7 +97074,7 @@
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>التبانة</t>
+          <t>الرمانة</t>
         </is>
       </c>
       <c r="C690" t="inlineStr">
@@ -97118,7 +97096,7 @@
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>الرمانة</t>
+          <t>الزاهرية</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
@@ -97140,7 +97118,7 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>الزاهرية</t>
+          <t>السويقه</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
@@ -97162,7 +97140,7 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>السويقه</t>
+          <t>القبة</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
@@ -97184,7 +97162,7 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>القبة</t>
+          <t>المهاترة</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
@@ -97206,7 +97184,7 @@
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>المهاترة</t>
+          <t>وادي النحلة</t>
         </is>
       </c>
       <c r="C695" t="inlineStr">
@@ -97215,28 +97193,6 @@
         </is>
       </c>
       <c r="D695" t="inlineStr">
-        <is>
-          <t>الشمال</t>
-        </is>
-      </c>
-    </row>
-    <row r="696">
-      <c r="A696" t="inlineStr">
-        <is>
-          <t>Arabic</t>
-        </is>
-      </c>
-      <c r="B696" t="inlineStr">
-        <is>
-          <t>وادي النحلة</t>
-        </is>
-      </c>
-      <c r="C696" t="inlineStr">
-        <is>
-          <t>مدينة طرابلس</t>
-        </is>
-      </c>
-      <c r="D696" t="inlineStr">
         <is>
           <t>الشمال</t>
         </is>

</xml_diff>